<commit_message>
feat: start phase 03 payment request persistence
</commit_message>
<xml_diff>
--- a/Back End/outputs/development-test-register/APS-Development-and-Test-Register.xlsx
+++ b/Back End/outputs/development-test-register/APS-Development-and-Test-Register.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Raeae4ee5736c45d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="Rad260e42e37346c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="R8402b6de8aa44598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="R848c20b4683a4cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="Rc694b13819824493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="Rdef41892892e4999"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="R413240d54b504d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R20b4b8f0eade44b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Register" sheetId="2" r:id="Ree48af0a341547d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development Log" sheetId="3" r:id="Rd6430c686bbf4858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="4" r:id="Ra58e6f7af0ce4456"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Executions" sheetId="5" r:id="R6e801b8fa4c64f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acceptance Matrix" sheetId="6" r:id="Raba58e7df7f14e04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="7" r:id="Rcab40dd863354cdc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -248,7 +248,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -259,7 +259,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -270,7 +270,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -281,7 +281,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -292,7 +292,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -303,7 +303,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -314,7 +314,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -325,7 +325,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -336,7 +336,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -347,7 +347,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -358,7 +358,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -369,7 +369,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -380,7 +380,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -391,7 +391,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -402,7 +402,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -413,7 +413,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -424,7 +424,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -446,7 +446,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +457,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -479,7 +479,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -490,7 +490,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +501,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -512,7 +512,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +523,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +534,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -545,7 +545,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -556,7 +556,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -567,7 +567,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -578,7 +578,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -589,7 +589,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -600,7 +600,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -611,7 +611,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -622,7 +622,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -633,7 +633,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -644,7 +644,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -655,7 +655,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF7EE"/>
         </x:patternFill>
       </x:fill>
@@ -666,7 +666,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -677,7 +677,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -688,7 +688,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -699,7 +699,7 @@
         <x:color rgb="FFB45309"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF7E6"/>
         </x:patternFill>
       </x:fill>
@@ -844,7 +844,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Red3e25e4d7a943f3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R72453ed2afd7404b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -897,7 +897,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestCaseTable" displayName="TestCaseTable" ref="A3:M23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TestCaseTable" displayName="TestCaseTable" ref="A3:M32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Phase"/>
@@ -1203,7 +1203,7 @@
       </x:c>
       <x:c r="B5" s="31" t="n">
         <x:f>COUNTIF('Phase Register'!$D$4:$D$13,"Validated")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
         <x:v>AG-P00-01</x:v>
@@ -1251,7 +1251,7 @@
       </x:c>
       <x:c r="B7" s="32" t="n">
         <x:f>COUNTIF('Test Cases'!$K$4:$K$200,"Passed")</x:f>
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
         <x:v>AG-P00-03</x:v>
@@ -1299,7 +1299,7 @@
       </x:c>
       <x:c r="B9" s="33" t="n">
         <x:f>COUNTIF('Test Cases'!$K$4:$K$200,"Not Run")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D9" s="23" t="str">
         <x:v>AG-P00-05</x:v>
@@ -1349,7 +1349,7 @@
       </x:c>
       <x:c r="E13" t="n">
         <x:f>COUNTIF('Test Cases'!$K$4:$K$200,D13)</x:f>
-        <x:v>20</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1367,7 +1367,7 @@
       </x:c>
       <x:c r="E15" t="n">
         <x:f>COUNTIF('Test Cases'!$K$4:$K$200,D15)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16"/>
@@ -1472,7 +1472,7 @@
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="Pending"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree69eda1a150448a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72ec412f90dd4e4d"/>
 </x:worksheet>
 </file>
 
@@ -1570,20 +1570,22 @@
         <x:v>Local auth, sessions, users, roles, permissions and authorization</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Validated</x:v>
       </x:c>
       <x:c r="E5" s="23" t="str">
         <x:v>Protected endpoints enforce identity, role and department boundaries</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
-        <x:v>PROJECT_MANIFEST.md</x:v>
-      </x:c>
-      <x:c r="G5" s="38"/>
+        <x:v>docs/phase-01-plan.md</x:v>
+      </x:c>
+      <x:c r="G5" s="38" t="n">
+        <x:v>46262</x:v>
+      </x:c>
       <x:c r="H5" s="23" t="str">
         <x:v>Backend Team</x:v>
       </x:c>
       <x:c r="I5" s="23" t="str">
-        <x:v>LifeOS SAML remains behind an adapter</x:v>
+        <x:v>Phase 01 local validation complete</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="120" hidden="0" customHeight="1">
@@ -1597,20 +1599,20 @@
         <x:v>Departments, cost centers, vendors, accounts, tax codes, currencies and payment methods</x:v>
       </x:c>
       <x:c r="D6" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Deferred</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
         <x:v>Reference data is persisted, validated and safely administered</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>PROJECT_MANIFEST.md</x:v>
+        <x:v>docs/phase-02-plan.md</x:v>
       </x:c>
       <x:c r="G6" s="38"/>
       <x:c r="H6" s="23" t="str">
         <x:v>Backend Team</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>Sensitive bank details encrypted and masked</x:v>
+        <x:v>Deferred by owner; may resume later</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="96" hidden="0" customHeight="1">
@@ -1624,20 +1626,22 @@
         <x:v>Drafts, request types, numbering, line items, allocations, submission and locking</x:v>
       </x:c>
       <x:c r="D7" s="23" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="E7" s="23" t="str">
         <x:v>Every request type persists and enforces ownership and totals</x:v>
       </x:c>
       <x:c r="F7" s="23" t="str">
-        <x:v>PROJECT_MANIFEST.md</x:v>
-      </x:c>
-      <x:c r="G7" s="38"/>
+        <x:v>docs/phase-03-plan.md</x:v>
+      </x:c>
+      <x:c r="G7" s="38" t="n">
+        <x:v>46273</x:v>
+      </x:c>
       <x:c r="H7" s="23" t="str">
         <x:v>Backend Team</x:v>
       </x:c>
       <x:c r="I7" s="23" t="str">
-        <x:v>Includes optimistic locking and duplicate checks</x:v>
+        <x:v>Core request persistence implemented; General Payment rules pending Finance confirmation</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="96" hidden="0" customHeight="1">
@@ -1823,7 +1827,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0395f250cc643f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R932ab9f7ddb443fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2409,7 +2413,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red06f90eb5f04b30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc56f4ed0b5254142"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3302,6 +3306,375 @@
       </x:c>
       <x:c r="M23" s="24" t="str">
         <x:v>Log contained method, path, status, duration_ms and request_id</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>TC-P03-001</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Request draft CRUD</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>API</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>Test database migrated and seeded</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>Create and retrieve an owned request draft</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Draft persists with request, line, amount and currency</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>pytest tests/test_payment_requests.py</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>Local isolated PostgreSQL run 2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>TC-P03-002</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Single-currency enforcement</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Negative</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>PHP request with USD line</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>POST /api/v1/requests</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>HTTP 422; mixed currency is rejected</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I25" t="str">
+        <x:v>pytest tests/test_payment_requests.py::test_mixed_currency_rejected_and_visibility_enforced</x:v>
+      </x:c>
+      <x:c r="J25" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K25" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>Amount and ISO currency pairs validated server-side</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>TC-P03-003</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Optimistic locking</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Concurrency</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>Existing draft at version 1</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Update twice with the same version</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>First update succeeds; stale update returns HTTP 409</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>pytest tests/test_payment_requests.py::test_request_crud_optimistic_lock_and_idempotent_submit</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K26" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L26" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M26" t="str">
+        <x:v>Local isolated PostgreSQL run 2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>TC-P03-004</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Idempotent submission and numbering</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Integration</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>Valid persisted draft</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>Submit twice with one idempotency key</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>One PR-2026-six-digit number is returned both times</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I27" t="str">
+        <x:v>pytest tests/test_payment_requests.py::test_request_crud_optimistic_lock_and_idempotent_submit</x:v>
+      </x:c>
+      <x:c r="J27" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K27" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L27" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M27" t="str">
+        <x:v>Calendar-year sequence stored transactionally</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>TC-P03-005</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Request visibility</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Security</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>Requests owned by users in different departments</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>Read another user's request without scope</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>HTTP 404 prevents unauthorized disclosure</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I28" t="str">
+        <x:v>pytest tests/test_payment_requests.py::test_mixed_currency_rejected_and_visibility_enforced</x:v>
+      </x:c>
+      <x:c r="J28" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K28" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L28" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M28" t="str">
+        <x:v>Owner/department/all scopes implemented</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>TC-P03-006</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Return for information</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>Workflow</x:v>
+      </x:c>
+      <x:c r="E29" t="str">
+        <x:v>Submitted Marketing request</x:v>
+      </x:c>
+      <x:c r="F29" t="str">
+        <x:v>Department Head returns with a note</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>Status becomes returned and immutable history is recorded</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I29" t="str">
+        <x:v>pytest tests/test_payment_requests.py::test_department_head_can_return_submitted_department_request</x:v>
+      </x:c>
+      <x:c r="J29" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K29" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L29" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M29" t="str">
+        <x:v>Local isolated PostgreSQL run 2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>TC-P03-007</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Backend regression suite</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>Test database at Alembic head</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>Run full pytest suite</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>All backend tests pass</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I30" t="str">
+        <x:v>pytest -q</x:v>
+      </x:c>
+      <x:c r="J30" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K30" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L30" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M30" t="str">
+        <x:v>36 passed; 1 warning; 2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>TC-P03-008</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Frontend production build</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>Build</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>Node dependencies installed</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>Run pnpm build</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>TypeScript and Vite production bundle succeed</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="I31" t="str">
+        <x:v>pnpm run build</x:v>
+      </x:c>
+      <x:c r="J31" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="K31" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="L31" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M31" t="str">
+        <x:v>Vite 7.3.6 build passed 2026-09-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>TC-P03-009</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>P03</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>General Payment business rules</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>Business validation</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>Finance-approved final rules available</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>Validate General Payment fields and documents</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>Current General Payment UI retained; final detailed rules approved</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="I32" t="str">
+        <x:v>Pending Finance confirmation</x:v>
+      </x:c>
+      <x:c r="J32" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="K32" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L32" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M32" t="str">
+        <x:v>Pending due ambiguous P.O. wording in source sheet</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3331,7 +3704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b1967dda4a4447b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15eaa0d36c464c35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4149,7 +4522,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6cf59bdbc114652"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfe03514fec4df5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4425,7 +4798,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670810af04834119"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R502a80a0a82b4de9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4675,6 +5048,6 @@
     <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6ff0f67d1094366"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41532ca1585d4dab"/>
 </x:worksheet>
 </file>
</xml_diff>